<commit_message>
NPB自動更新(1軍): 2026-09-01 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-01.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-01.xlsx
@@ -100619,7 +100619,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5回裏に先制3ラン、7回裏にもソロを放ち、1試合2本塁打4打点の大活躍。</t>
+          <t>5回に先制3ラン、7回にもソロを放ち、計2本塁打4打点と打線を牽引した。</t>
         </is>
       </c>
     </row>
@@ -100644,7 +100644,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>9回裏にサヨナラ犠牲フライを放ち、劇的な勝利を呼び込んだ。</t>
+          <t>9回裏1死二三塁のチャンスでサヨナラ犠牲フライを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -100669,7 +100669,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7回を無失点に抑え、8奪三振の快投で相手打線を完全に封じ込めた。</t>
+          <t>7回を被安打2、8奪三振無失点の快投で、相手打線を完全に封じ込めた。</t>
         </is>
       </c>
     </row>
@@ -100694,7 +100694,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6回を無失点に抑え、8奪三振の力投で試合を支配し、チームの勝利に貢献。</t>
+          <t>6回を被安打4、8奪三振無失点と圧巻の投球で、試合を支配し勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -100719,7 +100719,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回表に走者一掃のタイムリーツーベースを放ち、試合の流れを決定づけた。</t>
+          <t>7回表に走者一掃のタイムリーツーベースを放ち、一気に試合の流れを引き寄せた。</t>
         </is>
       </c>
     </row>
@@ -100734,17 +100734,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>床田 寛樹</t>
+          <t>カストロ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>日本ハム</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>8回を投げ1失点と好投し、試合の主導権を握り続けた。</t>
+          <t>8回裏に勝ち越しタイムリーヒットを放ち、接戦を制する貴重な一打となった。</t>
         </is>
       </c>
     </row>

</xml_diff>